<commit_message>
wip(feature): snapshot current 2.0.0 worktree state
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/opentherm specification/OT specification 2.3b.xlsx
+++ b/docs/opentherm specification/OT specification 2.3b.xlsx
@@ -8,7 +8,6 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Robert\Documents\GitHub\Rvdb\OTGW-firmware\specification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{407B3066-18E9-48D3-B950-7556F5DAE4A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="11190"/>
   </bookViews>
@@ -3945,4 +3944,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7efabe30-8cd7-44ff-a516-5db03a0430e7}" enabled="1" method="Standard" siteId="{c8fba477-6d4d-4f00-941a-6e6150c721f3}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>